<commit_message>
Soluciono problema en data missing y pruebo cronjob de mnm.py
</commit_message>
<xml_diff>
--- a/github_actions/update_workflow/schedules.xlsx
+++ b/github_actions/update_workflow/schedules.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,46 +451,35 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>45431.5</v>
+        <v>45458.75</v>
       </c>
       <c r="B2" t="n">
-        <v>48</v>
+        <v>6</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45431.48958333334</v>
+        <v>45458.73958333334</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45430.4375</v>
+        <v>45458.85416666666</v>
       </c>
       <c r="B3" t="n">
-        <v>59</v>
+        <v>6</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45430.42708333334</v>
+        <v>45458.84375</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45431.66666666666</v>
+        <v>45459.54166666666</v>
       </c>
       <c r="B4" t="n">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45431.65625</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>45438.65625</v>
-      </c>
-      <c r="B5" t="n">
-        <v>77</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>45438.64583333334</v>
+        <v>45459.53125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>